<commit_message>
Add LTM (Last Twelve Months) data to all visualizations and analysis
Updated all data visualizations and reports to include most recent LTM periods:

Cummins Power Systems LTM (Q3'24-Q2'25):
- Revenue: $6.9B (+7.6% vs 2024)
- EBITDA: $1.46B
- EBITDA Margin: 21.2% (NEW HIGH - leads Caterpillar by 1.3 pts!)

Caterpillar Energy & Transportation LTM (Q4'24-Q3'25):
- Revenue: $30.5B (+5.5% vs 2024)
- Operating Profit: $6.05B
- Operating Margin: 19.9%

Key updates:
✅ Visualization now shows 2019-2024 + LTM data point
✅ All 4 charts updated with LTM period
✅ Margin improvement now 16.0 pts for Cummins (5.2% → 21.2%)
✅ Excel file updated with latest LTM-inclusive PNG
✅ Summary insights show Cummins margin leadership

Cummins Power Systems has achieved superior profitability vs Caterpillar for the first time, with LTM margin of 21.2% vs 19.9%, despite being 4.4x smaller by revenue.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Power_Systems_Comparison.xlsx
+++ b/Power_Systems_Comparison.xlsx
@@ -941,7 +941,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="36294060" cy="26951940"/>
+    <ext cx="36294060" cy="27020520"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2420,7 +2420,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>- Report Generated: October 29, 2025</t>
+          <t>- Report Generated: October 30, 2025</t>
         </is>
       </c>
     </row>

</xml_diff>